<commit_message>
Improve launch archive and member access flows
</commit_message>
<xml_diff>
--- a/content/member-assets/cafe-menu-refresh-package/menu-refresh-pricing-sheet.xlsx
+++ b/content/member-assets/cafe-menu-refresh-package/menu-refresh-pricing-sheet.xlsx
@@ -17,10 +17,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0%"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -77,7 +78,7 @@
       </bottom>
     </border>
   </borders>
-  <cellXfs count="6">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -96,7 +97,49 @@
     <xf numFmtId="166" fontId="2" fillId="3" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="3" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEAF8F0"/>
+        </patternFill>
+      </fill>
+      <font>
+        <color rgb="FF0F6B3F"/>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF4E8"/>
+        </patternFill>
+      </fill>
+      <font>
+        <color rgb="FF8A4B00"/>
+        <b/>
+      </font>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
@@ -107,10 +150,8 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="52" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="8" width="24" customWidth="1"/>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="2" width="58" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -119,19 +160,14 @@
           <t>Side Hustle Stephen - The Launchpad</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="1">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="A2" t="inlineStr" s="2">
+      <c r="A2" t="inlineStr" s="6">
         <is>
           <t>Asset</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="2">
+      <c r="B2" t="inlineStr" s="6">
         <is>
           <t>Menu Refresh Pricing Sheet</t>
         </is>
@@ -150,12 +186,12 @@
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" t="inlineStr" s="2">
+      <c r="A4" t="inlineStr" s="6">
         <is>
           <t>What this is</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr" s="2">
+      <c r="B4" t="inlineStr" s="6">
         <is>
           <t>Starter, standard, and retainer pricing ladder.</t>
         </is>
@@ -174,12 +210,12 @@
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" t="inlineStr" s="2">
+      <c r="A6" t="inlineStr" s="6">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr" s="2">
+      <c r="B6" t="inlineStr" s="6">
         <is>
           <t>Local Service</t>
         </is>
@@ -198,12 +234,12 @@
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" t="inlineStr" s="2">
+      <c r="A8" t="inlineStr" s="6">
         <is>
           <t>Time to first sale</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr" s="2">
+      <c r="B8" t="inlineStr" s="6">
         <is>
           <t>1-7 days</t>
         </is>
@@ -222,12 +258,12 @@
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
-      <c r="A10" t="inlineStr" s="2">
+      <c r="A10" t="inlineStr" s="6">
         <is>
           <t>How to use</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr" s="2">
+      <c r="B10" t="inlineStr" s="6">
         <is>
           <t>Work left to right through the tabs. Replace the sample values, keep the formulas, and verify every fact before client use.</t>
         </is>
@@ -246,9 +282,12 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B11"/>
   <pageMargins left="0.45" right="0.45" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddHeader>&amp;LSide Hustle Stephen - Start Here&amp;R&amp;D</oddHeader>
+    <oddFooter>&amp;LVerify facts before client use&amp;RPage &amp;P of &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -259,10 +298,8 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="52" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="8" width="24" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="58" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -278,10 +315,10 @@
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="A2" s="4">
+      <c r="A2" s="8">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr" s="2">
+      <c r="B2" t="inlineStr" s="6">
         <is>
           <t>Update the Pricing Ladder with your local market prices and delivery scope.</t>
         </is>
@@ -298,10 +335,10 @@
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="4">
+      <c r="A4" s="8">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr" s="2">
+      <c r="B4" t="inlineStr" s="6">
         <is>
           <t>Use Retainer Tracker monthly to monitor included refreshes and extra revenue.</t>
         </is>
@@ -318,9 +355,12 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B5"/>
   <pageMargins left="0.45" right="0.45" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddHeader>&amp;LSide Hustle Stephen - Instructions&amp;R&amp;D</oddHeader>
+    <oddFooter>&amp;LVerify facts before client use&amp;RPage &amp;P of &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -331,10 +371,11 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="52" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="8" width="24" customWidth="1"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="58" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
+    <col min="5" max="5" width="38" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -365,23 +406,23 @@
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="A2" t="inlineStr" s="2">
+      <c r="A2" t="inlineStr" s="6">
         <is>
           <t>Starter Refresh</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="2">
+      <c r="B2" t="inlineStr" s="6">
         <is>
           <t>1 print menu + 1 Instagram menu panel</t>
         </is>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="7">
         <v>149</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="7">
         <v>0</v>
       </c>
-      <c r="E2" t="inlineStr" s="2">
+      <c r="E2" t="inlineStr" s="6">
         <is>
           <t>Tiny cafes testing demand</t>
         </is>
@@ -411,23 +452,23 @@
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" t="inlineStr" s="2">
+      <c r="A4" t="inlineStr" s="6">
         <is>
           <t>Full Menu System</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr" s="2">
+      <c r="B4" t="inlineStr" s="6">
         <is>
           <t>Full redesign, QR flow, specials template, launch posts</t>
         </is>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="7">
         <v>699</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="7">
         <v>199</v>
       </c>
-      <c r="E4" t="inlineStr" s="2">
+      <c r="E4" t="inlineStr" s="6">
         <is>
           <t>Multi-location or high-change menus</t>
         </is>
@@ -457,23 +498,23 @@
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" t="inlineStr" s="2">
+      <c r="A6" t="inlineStr" s="6">
         <is>
           <t>Multi-location Add-on</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr" s="2">
+      <c r="B6" t="inlineStr" s="6">
         <is>
           <t>Replicate final system across each extra location</t>
         </is>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="7">
         <v>249</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="7">
         <v>75</v>
       </c>
-      <c r="E6" t="inlineStr" s="2">
+      <c r="E6" t="inlineStr" s="6">
         <is>
           <t>Small cafe groups</t>
         </is>
@@ -483,6 +524,10 @@
   <autoFilter ref="A1:E6"/>
   <pageMargins left="0.45" right="0.45" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddHeader>&amp;LSide Hustle Stephen - Pricing Ladder&amp;R&amp;D</oddHeader>
+    <oddFooter>&amp;LVerify facts before client use&amp;RPage &amp;P of &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -493,10 +538,8 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="52" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="8" width="24" customWidth="1"/>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -512,12 +555,12 @@
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="A2" t="inlineStr" s="2">
+      <c r="A2" t="inlineStr" s="6">
         <is>
           <t>Base package price</t>
         </is>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="7">
         <v>349</v>
       </c>
     </row>
@@ -532,12 +575,12 @@
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" t="inlineStr" s="2">
+      <c r="A4" t="inlineStr" s="6">
         <is>
           <t>Extra menu page count</t>
         </is>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="8">
         <v>2</v>
       </c>
     </row>
@@ -552,12 +595,12 @@
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" t="inlineStr" s="2">
+      <c r="A6" t="inlineStr" s="6">
         <is>
           <t>Extra social panels</t>
         </is>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="8">
         <v>3</v>
       </c>
     </row>
@@ -572,12 +615,12 @@
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" t="inlineStr" s="2">
+      <c r="A8" t="inlineStr" s="6">
         <is>
           <t>Estimated quote</t>
         </is>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="7">
         <f>B2+B3+(B4*B5)+(B6*B7)</f>
       </c>
     </row>
@@ -592,9 +635,12 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B9"/>
   <pageMargins left="0.45" right="0.45" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddHeader>&amp;LSide Hustle Stephen - Quote Builder&amp;R&amp;D</oddHeader>
+    <oddFooter>&amp;LVerify facts before client use&amp;RPage &amp;P of &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -605,10 +651,12 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="52" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="8" width="24" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -644,26 +692,26 @@
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="A2" t="inlineStr" s="2">
+      <c r="A2" t="inlineStr" s="6">
         <is>
           <t>July</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="2">
+      <c r="B2" t="inlineStr" s="6">
         <is>
           <t>Example Cafe</t>
         </is>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="8">
         <v>2</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="8">
         <v>3</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="7">
         <v>45</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="7">
         <f>MAX(0,D2-C2)*E2</f>
       </c>
     </row>
@@ -692,33 +740,36 @@
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" t="inlineStr" s="2">
+      <c r="A4" t="inlineStr" s="6">
         <is>
           <t>September</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr" s="2">
+      <c r="B4" t="inlineStr" s="6">
         <is>
           <t/>
         </is>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="8">
         <v>2</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="8">
         <v>0</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="7">
         <v>45</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="7">
         <f>MAX(0,D4-C4)*E4</f>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F4"/>
   <pageMargins left="0.45" right="0.45" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddHeader>&amp;LSide Hustle Stephen - Retainer Tracker&amp;R&amp;D</oddHeader>
+    <oddFooter>&amp;LVerify facts before client use&amp;RPage &amp;P of &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -729,10 +780,10 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="52" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="8" width="24" customWidth="1"/>
+    <col min="1" max="1" width="46" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -758,22 +809,22 @@
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="A2" t="inlineStr" s="2">
+      <c r="A2" t="inlineStr" s="6">
         <is>
           <t>Current menu file or photos</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="2">
+      <c r="B2" t="inlineStr" s="6">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr" s="2">
+      <c r="C2" t="inlineStr" s="6">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr" s="2">
+      <c r="D2" t="inlineStr" s="6">
         <is>
           <t>Open</t>
         </is>
@@ -802,22 +853,22 @@
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" t="inlineStr" s="2">
+      <c r="A4" t="inlineStr" s="6">
         <is>
           <t>Logo, fonts, brand colors</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr" s="2">
+      <c r="B4" t="inlineStr" s="6">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr" s="2">
+      <c r="C4" t="inlineStr" s="6">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr" s="2">
+      <c r="D4" t="inlineStr" s="6">
         <is>
           <t>Open</t>
         </is>
@@ -847,6 +898,28 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:D5"/>
+  <conditionalFormatting sqref="C2:C200">
+    <cfRule type="containsText" operator="containsText" text="Done" dxfId="0" priority="7">
+      <formula>NOT(ISERROR(SEARCH("Done",C2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" operator="containsText" text="Approved" dxfId="0" priority="8">
+      <formula>NOT(ISERROR(SEARCH("Approved",C2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" operator="containsText" text="Open" dxfId="1" priority="9">
+      <formula>NOT(ISERROR(SEARCH("Open",C2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D200">
+    <cfRule type="containsText" operator="containsText" text="Done" dxfId="0" priority="10">
+      <formula>NOT(ISERROR(SEARCH("Done",D2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" operator="containsText" text="Approved" dxfId="0" priority="11">
+      <formula>NOT(ISERROR(SEARCH("Approved",D2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" operator="containsText" text="Open" dxfId="1" priority="12">
+      <formula>NOT(ISERROR(SEARCH("Open",D2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="C2:C200">
       <formula1>"Open,In progress,Done,Yes,No,Approved"</formula1>
@@ -857,6 +930,10 @@
   </dataValidations>
   <pageMargins left="0.45" right="0.45" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddHeader>&amp;LSide Hustle Stephen - Client Inputs&amp;R&amp;D</oddHeader>
+    <oddFooter>&amp;LVerify facts before client use&amp;RPage &amp;P of &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -867,10 +944,8 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="52" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="8" width="24" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="58" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -886,12 +961,12 @@
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="A2" t="inlineStr" s="2">
+      <c r="A2" t="inlineStr" s="6">
         <is>
           <t>Scope</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="2">
+      <c r="B2" t="inlineStr" s="6">
         <is>
           <t>I will refresh your customer-facing menu assets across the agreed formats and return final files ready to use.</t>
         </is>
@@ -910,21 +985,24 @@
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" t="inlineStr" s="2">
+      <c r="A4" t="inlineStr" s="6">
         <is>
           <t>Not included</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr" s="2">
+      <c r="B4" t="inlineStr" s="6">
         <is>
           <t>Photography, new brand identity, paid ads, printing costs, and menu engineering are not included unless scoped separately.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B4"/>
   <pageMargins left="0.45" right="0.45" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddHeader>&amp;LSide Hustle Stephen - Proposal Copy&amp;R&amp;D</oddHeader>
+    <oddFooter>&amp;LVerify facts before client use&amp;RPage &amp;P of &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -936,9 +1014,8 @@
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="52" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="8" width="24" customWidth="1"/>
+    <col min="2" max="2" width="58" customWidth="1"/>
+    <col min="3" max="3" width="58" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -959,17 +1036,17 @@
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="A2" t="inlineStr" s="2">
+      <c r="A2" t="inlineStr" s="6">
         <is>
           <t>Asset</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="2">
+      <c r="B2" t="inlineStr" s="6">
         <is>
           <t>Menu Refresh Pricing Sheet</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr" s="2">
+      <c r="C2" t="inlineStr" s="6">
         <is>
           <t>Use this as the named deliverable in the proposal and handoff.</t>
         </is>
@@ -993,17 +1070,17 @@
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" t="inlineStr" s="2">
+      <c r="A4" t="inlineStr" s="6">
         <is>
           <t>Priority decision</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr" s="2">
+      <c r="B4" t="inlineStr" s="6">
         <is>
           <t>Standard package should include the formats most cafes actually use: print, Instagram, QR, and Google menu link.</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr" s="2">
+      <c r="C4" t="inlineStr" s="6">
         <is>
           <t>Use this to keep the delivery focused.</t>
         </is>
@@ -1027,17 +1104,17 @@
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" t="inlineStr" s="2">
+      <c r="A6" t="inlineStr" s="6">
         <is>
           <t>Upsell path</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr" s="2">
+      <c r="B6" t="inlineStr" s="6">
         <is>
           <t>Raise price when there are multiple locations, poor source files, rush turnaround, or more than one approval stakeholder.</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr" s="2">
+      <c r="C6" t="inlineStr" s="6">
         <is>
           <t>Use after the first asset is approved.</t>
         </is>
@@ -1047,6 +1124,10 @@
   <autoFilter ref="A1:C6"/>
   <pageMargins left="0.45" right="0.45" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddHeader>&amp;LSide Hustle Stephen - Worked Example&amp;R&amp;D</oddHeader>
+    <oddFooter>&amp;LVerify facts before client use&amp;RPage &amp;P of &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1057,10 +1138,10 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="52" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="8" width="24" customWidth="1"/>
+    <col min="1" max="1" width="56" customWidth="1"/>
+    <col min="2" max="2" width="58" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1086,22 +1167,22 @@
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="A2" t="inlineStr" s="2">
+      <c r="A2" t="inlineStr" s="6">
         <is>
           <t>1. Collect</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr" s="2">
+      <c r="B2" t="inlineStr" s="6">
         <is>
           <t>Gather source material and visible proof before editing.</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr" s="2">
+      <c r="C2" t="inlineStr" s="6">
         <is>
           <t>You</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr" s="2">
+      <c r="D2" t="inlineStr" s="6">
         <is>
           <t>Open</t>
         </is>
@@ -1130,22 +1211,22 @@
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" t="inlineStr" s="2">
+      <c r="A4" t="inlineStr" s="6">
         <is>
           <t>3. Flag</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr" s="2">
+      <c r="B4" t="inlineStr" s="6">
         <is>
           <t>Mark every uncertain fact, price, or claim for client approval.</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr" s="2">
+      <c r="C4" t="inlineStr" s="6">
         <is>
           <t>You</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr" s="2">
+      <c r="D4" t="inlineStr" s="6">
         <is>
           <t>Open</t>
         </is>
@@ -1174,22 +1255,22 @@
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" t="inlineStr" s="2">
+      <c r="A6" t="inlineStr" s="6">
         <is>
           <t>5. Deliver</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr" s="2">
+      <c r="B6" t="inlineStr" s="6">
         <is>
           <t>Send working file, final export, and a summary of what changed.</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr" s="2">
+      <c r="C6" t="inlineStr" s="6">
         <is>
           <t>You</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr" s="2">
+      <c r="D6" t="inlineStr" s="6">
         <is>
           <t>Open</t>
         </is>
@@ -1218,22 +1299,22 @@
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" t="inlineStr" s="2">
+      <c r="A8" t="inlineStr" s="6">
         <is>
           <t>QA - placeholders removed or marked</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr" s="2">
+      <c r="B8" t="inlineStr" s="6">
         <is>
           <t>Required before sending</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr" s="2">
+      <c r="C8" t="inlineStr" s="6">
         <is>
           <t>You</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr" s="2">
+      <c r="D8" t="inlineStr" s="6">
         <is>
           <t>Open</t>
         </is>
@@ -1262,22 +1343,22 @@
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
-      <c r="A10" t="inlineStr" s="2">
+      <c r="A10" t="inlineStr" s="6">
         <is>
           <t>QA - no guaranteed revenue/ranking/performance claims</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr" s="2">
+      <c r="B10" t="inlineStr" s="6">
         <is>
           <t>Required before sending</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr" s="2">
+      <c r="C10" t="inlineStr" s="6">
         <is>
           <t>You</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr" s="2">
+      <c r="D10" t="inlineStr" s="6">
         <is>
           <t>Open</t>
         </is>
@@ -1307,6 +1388,17 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:D11"/>
+  <conditionalFormatting sqref="D2:D200">
+    <cfRule type="containsText" operator="containsText" text="Done" dxfId="0" priority="10">
+      <formula>NOT(ISERROR(SEARCH("Done",D2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" operator="containsText" text="Approved" dxfId="0" priority="11">
+      <formula>NOT(ISERROR(SEARCH("Approved",D2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" operator="containsText" text="Open" dxfId="1" priority="12">
+      <formula>NOT(ISERROR(SEARCH("Open",D2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="D2:D200">
       <formula1>"Open,In progress,Done,Yes,No,Approved"</formula1>
@@ -1314,5 +1406,9 @@
   </dataValidations>
   <pageMargins left="0.45" right="0.45" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddHeader>&amp;LSide Hustle Stephen - Delivery &amp; QA&amp;R&amp;D</oddHeader>
+    <oddFooter>&amp;LVerify facts before client use&amp;RPage &amp;P of &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Remove fake proof and fix archive search
</commit_message>
<xml_diff>
--- a/content/member-assets/cafe-menu-refresh-package/menu-refresh-pricing-sheet.xlsx
+++ b/content/member-assets/cafe-menu-refresh-package/menu-refresh-pricing-sheet.xlsx
@@ -185,7 +185,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="54" customHeight="1">
       <c r="A4" t="inlineStr" s="6">
         <is>
           <t>What this is</t>
@@ -193,7 +193,7 @@
       </c>
       <c r="B4" t="inlineStr" s="6">
         <is>
-          <t>Starter, standard, and retainer pricing ladder.</t>
+          <t>Starter, full-refresh, and retainer pricing with a delivery-time and private-floor quote check.</t>
         </is>
       </c>
     </row>
@@ -257,7 +257,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="42" customHeight="1">
+    <row r="10" ht="54" customHeight="1">
       <c r="A10" t="inlineStr" s="6">
         <is>
           <t>How to use</t>
@@ -269,7 +269,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1">
+    <row r="11" ht="54" customHeight="1">
       <c r="A11" t="inlineStr" s="2">
         <is>
           <t>Delivery standards</t>
@@ -314,7 +314,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="54" customHeight="1">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -324,7 +324,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
+    <row r="3" ht="54" customHeight="1">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -334,7 +334,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="54" customHeight="1">
       <c r="A4" s="8">
         <v>3</v>
       </c>
@@ -440,10 +440,10 @@
         </is>
       </c>
       <c r="C3" s="3">
-        <v>349</v>
+        <v>449</v>
       </c>
       <c r="D3" s="3">
-        <v>99</v>
+        <v>175</v>
       </c>
       <c r="E3" t="inlineStr" s="2">
         <is>
@@ -454,19 +454,19 @@
     <row r="4" ht="42" customHeight="1">
       <c r="A4" t="inlineStr" s="6">
         <is>
-          <t>Full Menu System</t>
+          <t>Full Menu Refresh</t>
         </is>
       </c>
       <c r="B4" t="inlineStr" s="6">
         <is>
-          <t>Full redesign, QR flow, specials template, launch posts</t>
+          <t>Bounded menu refresh, QR flow, specials template, launch posts</t>
         </is>
       </c>
       <c r="C4" s="7">
         <v>699</v>
       </c>
       <c r="D4" s="7">
-        <v>199</v>
+        <v>275</v>
       </c>
       <c r="E4" t="inlineStr" s="6">
         <is>
@@ -489,7 +489,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="3">
-        <v>149</v>
+        <v>225</v>
       </c>
       <c r="E5" t="inlineStr" s="2">
         <is>
@@ -505,14 +505,14 @@
       </c>
       <c r="B6" t="inlineStr" s="6">
         <is>
-          <t>Replicate final system across each extra location</t>
+          <t>Adapt the approved refresh across each extra location</t>
         </is>
       </c>
       <c r="C6" s="7">
         <v>249</v>
       </c>
       <c r="D6" s="7">
-        <v>75</v>
+        <v>150</v>
       </c>
       <c r="E6" t="inlineStr" s="6">
         <is>
@@ -538,8 +538,8 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
-    <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="1" max="1" width="29" customWidth="1"/>
+    <col min="2" max="2" width="27" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -561,77 +561,137 @@
         </is>
       </c>
       <c r="B2" s="7">
-        <v>349</v>
+        <v>449</v>
       </c>
     </row>
     <row r="3" ht="42" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
-          <t>Rush fee</t>
-        </is>
-      </c>
-      <c r="B3" s="3">
-        <v>75</v>
+          <t>Estimated delivery hours</t>
+        </is>
+      </c>
+      <c r="B3" s="4">
+        <v>6</v>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" t="inlineStr" s="6">
         <is>
-          <t>Extra menu page count</t>
-        </is>
-      </c>
-      <c r="B4" s="8">
-        <v>2</v>
+          <t>Private hourly price floor</t>
+        </is>
+      </c>
+      <c r="B4" s="7">
+        <v>60</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" t="inlineStr" s="2">
         <is>
-          <t>Price per extra page</t>
+          <t>Direct costs</t>
         </is>
       </c>
       <c r="B5" s="3">
-        <v>35</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" t="inlineStr" s="6">
         <is>
-          <t>Extra social panels</t>
-        </is>
-      </c>
-      <c r="B6" s="8">
-        <v>3</v>
+          <t>Risk buffer rate</t>
+        </is>
+      </c>
+      <c r="B6" s="9">
+        <v>0.1</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
       <c r="A7" t="inlineStr" s="2">
         <is>
-          <t>Price per social panel</t>
+          <t>Rush fee</t>
         </is>
       </c>
       <c r="B7" s="3">
-        <v>25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" t="inlineStr" s="6">
         <is>
-          <t>Estimated quote</t>
-        </is>
-      </c>
-      <c r="B8" s="7">
-        <f>B2+B3+(B4*B5)+(B6*B7)</f>
+          <t>Extra menu page count</t>
+        </is>
+      </c>
+      <c r="B8" s="8">
+        <v>0</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" t="inlineStr" s="2">
         <is>
+          <t>Price per extra page</t>
+        </is>
+      </c>
+      <c r="B9" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" t="inlineStr" s="6">
+        <is>
+          <t>Extra social panels</t>
+        </is>
+      </c>
+      <c r="B10" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" t="inlineStr" s="2">
+        <is>
+          <t>Price per social panel</t>
+        </is>
+      </c>
+      <c r="B11" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" t="inlineStr" s="6">
+        <is>
+          <t>Scope-based quote subtotal</t>
+        </is>
+      </c>
+      <c r="B12" s="7">
+        <f>B2+B7+(B8*B9)+(B10*B11)</f>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" t="inlineStr" s="2">
+        <is>
+          <t>Private minimum</t>
+        </is>
+      </c>
+      <c r="B13" s="4">
+        <f>(B3*B4)+B5</f>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" t="inlineStr" s="6">
+        <is>
+          <t>Recommended quote</t>
+        </is>
+      </c>
+      <c r="B14" s="7">
+        <f>MAX(B12,B13)*(1+B6)</f>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" t="inlineStr" s="2">
+        <is>
           <t>Deposit due at 50%</t>
         </is>
       </c>
-      <c r="B9" s="3">
-        <f>B8*0.5</f>
+      <c r="B15" s="3">
+        <f>B14*0.5</f>
       </c>
     </row>
   </sheetData>
@@ -960,7 +1020,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="54" customHeight="1">
       <c r="A2" t="inlineStr" s="6">
         <is>
           <t>Scope</t>
@@ -972,7 +1032,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
+    <row r="3" ht="54" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
           <t>Approval</t>
@@ -984,7 +1044,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="54" customHeight="1">
       <c r="A4" t="inlineStr" s="6">
         <is>
           <t>Not included</t>
@@ -1052,7 +1112,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
+    <row r="3" ht="54" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
           <t>Prospect context</t>
@@ -1069,7 +1129,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="54" customHeight="1">
       <c r="A4" t="inlineStr" s="6">
         <is>
           <t>Priority decision</t>
@@ -1086,7 +1146,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="54" customHeight="1">
       <c r="A5" t="inlineStr" s="2">
         <is>
           <t>Approval point</t>
@@ -1103,7 +1163,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
+    <row r="6" ht="54" customHeight="1">
       <c r="A6" t="inlineStr" s="6">
         <is>
           <t>Upsell path</t>
@@ -1188,7 +1248,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
+    <row r="3" ht="54" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
           <t>2. Draft</t>
@@ -1210,7 +1270,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="54" customHeight="1">
       <c r="A4" t="inlineStr" s="6">
         <is>
           <t>3. Flag</t>
@@ -1232,7 +1292,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="54" customHeight="1">
       <c r="A5" t="inlineStr" s="2">
         <is>
           <t>4. Approve</t>
@@ -1254,7 +1314,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
+    <row r="6" ht="54" customHeight="1">
       <c r="A6" t="inlineStr" s="6">
         <is>
           <t>5. Deliver</t>

</xml_diff>